<commit_message>
fix: drop per-company subtotals and total from 창원공동물류센터 export
Only title, header, and data rows, matching the original sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/lib/excel-templates/files/changwon.xlsx
+++ b/app/lib/excel-templates/files/changwon.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">'2024.02'!$B$3:$I$416</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'2024.02'!$A1:$I6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'2024.02'!$A1:$I4</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
@@ -114,7 +114,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -152,24 +152,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -209,18 +196,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -684,34 +659,8 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
     </row>
-    <row r="5" ht="24.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-    </row>
-    <row r="6" ht="24.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25"/>
@@ -1115,8 +1064,8 @@
     <row r="407" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="408" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="409" spans="1:16" x14ac:dyDescent="0.25"/>
-    <row r="410" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="411" spans="1:16" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="410" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="411" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="412" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="413" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="414" spans="1:16" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
feat: 창원공동물류센터 export summary block; unify 조은 as 에이큐
- Add bottom summary like the original sheet (rows 350-364): per-company
  totals, 공급가액, 부가세 10%, and grand totals, no extra labels
- Replace 조은 with 에이큐 in company options and the 창원 group

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/lib/excel-templates/files/changwon.xlsx
+++ b/app/lib/excel-templates/files/changwon.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">'2024.02'!$B$3:$I$416</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'2024.02'!$A1:$I4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'2024.02'!$A1:$I8</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
@@ -114,7 +114,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -152,11 +152,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -196,6 +209,24 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -659,10 +690,62 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="24.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" ht="24.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" ht="24.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" ht="24.75" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+    </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25"/>
@@ -1064,8 +1147,8 @@
     <row r="407" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="408" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="409" spans="1:16" x14ac:dyDescent="0.25"/>
-    <row r="410" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="411" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="410" spans="1:16" s="20" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="411" spans="1:16" s="20" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="412" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="413" spans="1:16" x14ac:dyDescent="0.25"/>
     <row r="414" spans="1:16" x14ac:dyDescent="0.25"/>

</xml_diff>